<commit_message>
Update financial data in Taller_final.xlsx
</commit_message>
<xml_diff>
--- a/Taller_final.xlsx
+++ b/Taller_final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eafit-my.sharepoint.com/personal/darmendar_eafit_edu_co/Documents/MAF/Finanzas Corporativas/Taller final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidarmendariz/finanzas-corporativas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="764" documentId="13_ncr:1_{9A198AE5-DFB1-4B20-96FE-55380C251E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30E17729-1738-0C4A-8CDA-E2F8C3AA2AFC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2BC65EF-C6ED-C344-8350-33BA99DCCD94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20240" firstSheet="1" activeTab="10" xr2:uid="{4A5FEAB5-AF17-D144-BB0B-4790A386B114}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20240" activeTab="10" xr2:uid="{4A5FEAB5-AF17-D144-BB0B-4790A386B114}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="2" r:id="rId1"/>
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -2352,14 +2352,12 @@
     <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="42" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="42" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="172" fontId="20" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2375,12 +2373,14 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="42" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="172" fontId="20" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Comma" xfId="6" builtinId="3"/>
@@ -2645,34 +2645,34 @@
                 <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>-2195711924.9955101</c:v>
+                  <c:v>-1793478653.7849333</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5414741026.4728117</c:v>
+                  <c:v>6862201586.9203444</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7106394547.2652617</c:v>
+                  <c:v>8683790747.3030453</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9005404496.5502529</c:v>
+                  <c:v>10720217143.950525</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11137745768.895601</c:v>
+                  <c:v>12998272906.196072</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13529006405.409296</c:v>
+                  <c:v>15543929387.198647</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>16182203815.408293</c:v>
+                  <c:v>18357655711.156792</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>19172528835.372379</c:v>
+                  <c:v>21520522347.328396</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>22565041869.693596</c:v>
+                  <c:v>25100818510.761791</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>26394705688.86586</c:v>
+                  <c:v>29132766304.14537</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3062,34 +3062,34 @@
                 <c:formatCode>0.0\x</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>8.1286530415287981</c:v>
+                  <c:v>14.96471979451398</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>65.838542427979178</c:v>
+                  <c:v>78.617761323886896</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>87.755807934357804</c:v>
+                  <c:v>103.29684494837487</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>117.63261973378687</c:v>
+                  <c:v>136.743255629239</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>159.3923777326539</c:v>
+                  <c:v>183.25666315287984</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>219.7438275785882</c:v>
+                  <c:v>250.18309750589123</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>310.80697237045035</c:v>
+                  <c:v>350.77714791932891</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>459.6738798683748</c:v>
+                  <c:v>514.71499066288914</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>734.41710270278793</c:v>
+                  <c:v>816.50516372521986</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1779.915399049032</c:v>
+                  <c:v>1966.0518176842911</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3471,34 +3471,34 @@
                 <c:formatCode>0.0\x</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0.80895198682443781</c:v>
+                  <c:v>1.0653044900613822</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.494236405247559</c:v>
+                  <c:v>5.1106863155835649</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.2644910722477762</c:v>
+                  <c:v>4.9224288924288082</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.3754789785983643</c:v>
+                  <c:v>6.1481050730758042</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.7938153926541371</c:v>
+                  <c:v>7.705310216552598</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.6208663706453592</c:v>
+                  <c:v>9.7025466023144791</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>10.98309772194906</c:v>
+                  <c:v>12.274503363325364</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>14.13850832497668</c:v>
+                  <c:v>15.697996625822482</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>18.450503419735949</c:v>
+                  <c:v>20.362159977095107</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>14.502165921754102</c:v>
+                  <c:v>15.915731551638485</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3885,31 +3885,31 @@
                 <c:formatCode>0.0\x</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>5.550966462910953</c:v>
+                  <c:v>3.9749201466934818</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.6340329887364039</c:v>
+                  <c:v>0.53682484210639336</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.477059962457897</c:v>
+                  <c:v>0.40877809883829974</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.35539875043134411</c:v>
+                  <c:v>0.30780934218288158</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.26064928638597801</c:v>
+                  <c:v>0.22793441779244636</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.1866872178843462</c:v>
+                  <c:v>0.16468568885592963</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.12906548119843894</c:v>
+                  <c:v>0.11476053772556309</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>8.3859490787008661E-2</c:v>
+                  <c:v>7.5105725861286693E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.8497304908023432E-2</c:v>
+                  <c:v>4.3723075514740542E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -4292,34 +4292,34 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>3.5552954778061065E-2</c:v>
+                  <c:v>6.5754886223256911E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.81189287854670089</c:v>
+                  <c:v>0.9935691448714028</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1509994165403077</c:v>
+                  <c:v>1.398696739354045</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.6980512719201346</c:v>
+                  <c:v>2.0614052039292154</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.6965970399616053</c:v>
+                  <c:v>3.305657344133226</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.0051666692588759</c:v>
+                  <c:v>6.3788967054391819</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>15.230378912991371</c:v>
+                  <c:v>24.60250191963048</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-24.269563097624886</c:v>
+                  <c:v>-18.779593361439836</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-7.8931985349709581</c:v>
+                  <c:v>-7.7266983681312933</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-5.1322792624758007</c:v>
+                  <c:v>-5.2365998091655221</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4692,34 +4692,34 @@
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"_);_(@_)</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>1513250000</c:v>
+                  <c:v>2113250000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11923669800</c:v>
+                  <c:v>14082805800</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14086279564.056005</c:v>
+                  <c:v>16439236884.504004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>16544796493.694756</c:v>
+                  <c:v>19102734044.070896</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>19336327637.347153</c:v>
+                  <c:v>22111623373.128967</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>22497523116.991997</c:v>
+                  <c:v>25503126769.407661</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>26033296965.235657</c:v>
+                  <c:v>29278357060.639275</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>30050265943.069538</c:v>
+                  <c:v>33552701489.819916</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>34641100225.799545</c:v>
+                  <c:v>38423646557.836823</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>39855490867.963867</c:v>
+                  <c:v>43939778486.000443</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5095,34 +5095,34 @@
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"_);_(@_)</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>-156488080.83863837</c:v>
+                  <c:v>-216488080.83863842</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-3494649548.1143785</c:v>
+                  <c:v>-3710563148.114378</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-4097371420.9662528</c:v>
+                  <c:v>-4332667153.0110521</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4773745405.0413704</c:v>
+                  <c:v>-5029539160.0789814</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-5532871174.7724819</c:v>
+                  <c:v>-5810400748.3506641</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-6383407714.9464569</c:v>
+                  <c:v>-6683968080.1880207</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-7324488314.407423</c:v>
+                  <c:v>-7648994323.9477835</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-8385001117.956502</c:v>
+                  <c:v>-8735244672.6315422</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-9588610068.1000595</c:v>
+                  <c:v>-9966864701.3037872</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-10948379136.027424</c:v>
+                  <c:v>-11356807897.831085</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5510,34 +5510,34 @@
                 <c:formatCode>0.0\x</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>-9.6700655531738402</c:v>
+                  <c:v>-9.7615073855965875</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-3.411978693667209</c:v>
+                  <c:v>-3.7953284280194919</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-3.4378820265052132</c:v>
+                  <c:v>-3.794253355713999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-3.4657894566858189</c:v>
+                  <c:v>-3.7981082234522097</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-3.4948089385331271</c:v>
+                  <c:v>-3.8055246670215572</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-3.5243750864158465</c:v>
+                  <c:v>-3.8155668105300493</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-3.554281998652058</c:v>
+                  <c:v>-3.827739415229189</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-3.5838117992276488</c:v>
+                  <c:v>-3.8410717440971203</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-3.612734273244206</c:v>
+                  <c:v>-3.8551387732604159</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-3.6403097091160173</c:v>
+                  <c:v>-3.8690254234547745</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5919,34 +5919,34 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0.15520512820512822</c:v>
+                  <c:v>0.21674358974358973</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.32701741654571842</c:v>
+                  <c:v>0.38623367198838898</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.34112810471835048</c:v>
+                  <c:v>0.39810978448393902</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.35465088371867143</c:v>
+                  <c:v>0.40948231141763392</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.36761107636676876</c:v>
+                  <c:v>0.42037339358652531</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3800328723064087</c:v>
+                  <c:v>0.43080415868768379</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.39193938081913327</c:v>
+                  <c:v>0.44079476960111491</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.40335268107635375</c:v>
+                  <c:v>0.45036447028165705</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4142938699583239</c:v>
+                  <c:v>0.45953162938229491</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.42478310756219528</c:v>
+                  <c:v>0.46831378172488458</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6334,34 +6334,34 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0.60653846153846158</c:v>
+                  <c:v>0.66807692307692312</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.64021044992743104</c:v>
+                  <c:v>0.69942670537010154</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.65187624941807931</c:v>
+                  <c:v>0.70885792918366786</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.66309252966181187</c:v>
+                  <c:v>0.7179239573607743</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.6738767800867127</c:v>
+                  <c:v>0.72663909730646925</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.68424580034409155</c:v>
+                  <c:v>0.7350170867253667</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.69421572802449438</c:v>
+                  <c:v>0.74307111680647608</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.70380206523235489</c:v>
+                  <c:v>0.75081385443765813</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.71301970406775894</c:v>
+                  <c:v>0.75825746349172995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.72188295106166223</c:v>
+                  <c:v>0.76541362522435141</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6743,34 +6743,34 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>7.3174358974358977E-2</c:v>
+                  <c:v>0.13471282051282052</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.30508217897705769</c:v>
+                  <c:v>0.3642984344197282</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.32175930993381924</c:v>
+                  <c:v>0.37874098969940778</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.33750653401897623</c:v>
+                  <c:v>0.39233796171793872</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.35240574139353087</c:v>
+                  <c:v>0.40516805861328742</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.36652248319868075</c:v>
+                  <c:v>0.4172937695799559</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.37989814312274206</c:v>
+                  <c:v>0.42875353190472371</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.39261728609063085</c:v>
+                  <c:v>0.43962907529593415</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.40472857800648554</c:v>
+                  <c:v>0.4499663374304565</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.4162587732225741</c:v>
+                  <c:v>0.45978944738526339</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7157,34 +7157,34 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>-1.6050059573193678E-2</c:v>
+                  <c:v>-2.2203905727039838E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-9.5843921051640191E-2</c:v>
+                  <c:v>-0.10176554659590724</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-9.9226239320703222E-2</c:v>
+                  <c:v>-0.10492440729726207</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.10232903300993026</c:v>
+                  <c:v>-0.10781217577982644</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-0.10518774640683672</c:v>
+                  <c:v>-0.11046397812881238</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-0.10782986004275938</c:v>
+                  <c:v>-0.11290698868088685</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.11027244911005209</c:v>
+                  <c:v>-0.11515798798825023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-0.11254851082394469</c:v>
+                  <c:v>-0.11724968974447506</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-0.11467598738898983</c:v>
+                  <c:v>-0.11919976333138693</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-0.11668872747240676</c:v>
+                  <c:v>-0.12104179488867572</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14756,10 +14756,10 @@
       <c r="H2" s="26"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B3" s="159" t="s">
+      <c r="B3" s="157" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="159"/>
+      <c r="C3" s="157"/>
       <c r="H3" s="26"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.2">
@@ -14978,7 +14978,7 @@
       <c r="D20" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="160" t="s">
+      <c r="E20" s="158" t="s">
         <v>30</v>
       </c>
     </row>
@@ -14992,7 +14992,7 @@
       <c r="D21" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="160"/>
+      <c r="E21" s="158"/>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
@@ -15004,7 +15004,7 @@
       <c r="D22" t="s">
         <v>34</v>
       </c>
-      <c r="E22" s="160"/>
+      <c r="E22" s="158"/>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
@@ -15013,7 +15013,7 @@
       <c r="C23" s="10">
         <v>0.02</v>
       </c>
-      <c r="E23" s="160"/>
+      <c r="E23" s="158"/>
     </row>
     <row r="24" spans="2:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
@@ -15039,7 +15039,7 @@
       <c r="D25" t="s">
         <v>40</v>
       </c>
-      <c r="E25" s="160" t="s">
+      <c r="E25" s="158" t="s">
         <v>41</v>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       <c r="D26" t="s">
         <v>43</v>
       </c>
-      <c r="E26" s="160"/>
+      <c r="E26" s="158"/>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
@@ -15065,17 +15065,17 @@
       <c r="D27" t="s">
         <v>43</v>
       </c>
-      <c r="E27" s="160"/>
+      <c r="E27" s="158"/>
     </row>
     <row r="28" spans="2:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="164">
+      <c r="C28" s="153">
         <v>30</v>
       </c>
       <c r="D28" s="39"/>
-      <c r="E28" s="160" t="s">
+      <c r="E28" s="158" t="s">
         <v>46</v>
       </c>
     </row>
@@ -15087,7 +15087,7 @@
         <v>90</v>
       </c>
       <c r="D29" s="39"/>
-      <c r="E29" s="160"/>
+      <c r="E29" s="158"/>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
@@ -15099,7 +15099,7 @@
       <c r="D30" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="160"/>
+      <c r="E30" s="158"/>
     </row>
     <row r="31" spans="2:5" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
@@ -15109,7 +15109,7 @@
         <v>0.06</v>
       </c>
       <c r="D31" s="11"/>
-      <c r="E31" s="160"/>
+      <c r="E31" s="158"/>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
@@ -15121,7 +15121,7 @@
       <c r="D32" t="s">
         <v>51</v>
       </c>
-      <c r="E32" s="160"/>
+      <c r="E32" s="158"/>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
@@ -15131,7 +15131,7 @@
         <v>0.02</v>
       </c>
       <c r="D33" s="39"/>
-      <c r="E33" s="160"/>
+      <c r="E33" s="158"/>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
@@ -15143,7 +15143,7 @@
       <c r="D34" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="E34" s="160"/>
+      <c r="E34" s="158"/>
     </row>
     <row r="35" spans="2:5" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
@@ -15155,7 +15155,7 @@
       <c r="D35" t="s">
         <v>56</v>
       </c>
-      <c r="E35" s="160"/>
+      <c r="E35" s="158"/>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
@@ -15616,44 +15616,44 @@
       </c>
       <c r="C9" s="135"/>
       <c r="D9" s="112">
-        <f>2000000</f>
-        <v>2000000</v>
+        <f>Datos!C22</f>
+        <v>1600000</v>
       </c>
       <c r="E9" s="112">
         <f>D9*(1+D4)*(1+Datos!$C$23)</f>
-        <v>2159136</v>
+        <v>1727308.8</v>
       </c>
       <c r="F9" s="112">
         <f>E9*(1+E4)*(1+Datos!$C$23)</f>
-        <v>2352957.320448</v>
+        <v>1882365.8563584001</v>
       </c>
       <c r="G9" s="112">
         <f>F9*(1+F4)*(1+Datos!$C$23)</f>
-        <v>2557937.550376148</v>
+        <v>2046350.0403009185</v>
       </c>
       <c r="H9" s="112">
         <f>G9*(1+G4)*(1+Datos!$C$23)</f>
-        <v>2775295.7357818112</v>
+        <v>2220236.5886254488</v>
       </c>
       <c r="I9" s="112">
         <f>H9*(1+H4)*(1+Datos!$C$23)</f>
-        <v>3005603.6524156649</v>
+        <v>2404482.9219325315</v>
       </c>
       <c r="J9" s="112">
         <f>I9*(1+I4)*(1+Datos!$C$23)</f>
-        <v>3245060.095403621</v>
+        <v>2596048.0763228964</v>
       </c>
       <c r="K9" s="112">
         <f>J9*(1+J4)*(1+Datos!$C$23)</f>
-        <v>3502435.5467503686</v>
+        <v>2801948.437400294</v>
       </c>
       <c r="L9" s="112">
         <f>K9*(1+K4)*(1+Datos!$C$23)</f>
-        <v>3782546.3320372761</v>
+        <v>3026037.0656298199</v>
       </c>
       <c r="M9" s="112">
         <f>L9*(1+L4)*(1+Datos!$C$23)</f>
-        <v>4084287.6180365537</v>
+        <v>3267430.094429242</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="13" x14ac:dyDescent="0.15">
@@ -15821,50 +15821,50 @@
     <row r="16" spans="1:14" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="110">
         <f t="shared" ref="A16:A37" si="1">D16/$D$15</f>
-        <v>0.30769230769230771</v>
+        <v>0.24615384615384617</v>
       </c>
       <c r="B16" s="122" t="s">
         <v>307</v>
       </c>
       <c r="D16" s="112">
         <f>D9*D10</f>
-        <v>3000000000</v>
+        <v>2400000000</v>
       </c>
       <c r="E16" s="112">
         <f t="shared" ref="E16:M16" si="2">E9*E10</f>
-        <v>10795680000</v>
+        <v>8636544000</v>
       </c>
       <c r="F16" s="112">
         <f t="shared" si="2"/>
-        <v>11764786602.24</v>
+        <v>9411829281.7919998</v>
       </c>
       <c r="G16" s="112">
         <f t="shared" si="2"/>
-        <v>12789687751.880739</v>
+        <v>10231750201.504593</v>
       </c>
       <c r="H16" s="112">
         <f t="shared" si="2"/>
-        <v>13876478678.909056</v>
+        <v>11101182943.127243</v>
       </c>
       <c r="I16" s="112">
         <f t="shared" si="2"/>
-        <v>15028018262.078325</v>
+        <v>12022414609.662657</v>
       </c>
       <c r="J16" s="112">
         <f t="shared" si="2"/>
-        <v>16225300477.018105</v>
+        <v>12980240381.614483</v>
       </c>
       <c r="K16" s="112">
         <f t="shared" si="2"/>
-        <v>17512177733.751842</v>
+        <v>14009742187.001471</v>
       </c>
       <c r="L16" s="112">
         <f t="shared" si="2"/>
-        <v>18912731660.186382</v>
+        <v>15130185328.149099</v>
       </c>
       <c r="M16" s="112">
         <f t="shared" si="2"/>
-        <v>20421438090.18277</v>
+        <v>16337150472.14621</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="13" x14ac:dyDescent="0.15">
@@ -15968,7 +15968,7 @@
     <row r="19" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="A19" s="110">
         <f t="shared" si="1"/>
-        <v>0.60653846153846158</v>
+        <v>0.66807692307692312</v>
       </c>
       <c r="B19" s="124" t="s">
         <v>310</v>
@@ -15976,43 +15976,43 @@
       <c r="C19" s="107"/>
       <c r="D19" s="120">
         <f>D15-D16-D17-D18</f>
-        <v>5913750000</v>
+        <v>6513750000</v>
       </c>
       <c r="E19" s="120">
         <f t="shared" ref="E19:M19" si="4">E15-E16-E17-E18</f>
-        <v>23343276600</v>
+        <v>25502412600</v>
       </c>
       <c r="F19" s="120">
         <f t="shared" si="4"/>
-        <v>26918072605.166405</v>
+        <v>29271029925.614403</v>
       </c>
       <c r="G19" s="120">
         <f t="shared" si="4"/>
-        <v>30933888687.125103</v>
+        <v>33491826237.501244</v>
       </c>
       <c r="H19" s="120">
         <f t="shared" si="4"/>
-        <v>35445891173.194046</v>
+        <v>38221186908.975861</v>
       </c>
       <c r="I19" s="120">
         <f t="shared" si="4"/>
-        <v>40506589910.29155</v>
+        <v>43512193562.707214</v>
       </c>
       <c r="J19" s="120">
         <f t="shared" si="4"/>
-        <v>46111018922.946358</v>
+        <v>49356079018.349976</v>
       </c>
       <c r="K19" s="120">
         <f t="shared" si="4"/>
-        <v>52434110949.941345</v>
+        <v>55936546496.691719</v>
       </c>
       <c r="L19" s="120">
         <f t="shared" si="4"/>
-        <v>59619001927.462395</v>
+        <v>63401548259.49968</v>
       </c>
       <c r="M19" s="120">
         <f t="shared" si="4"/>
-        <v>67731034618.800926</v>
+        <v>71815322236.837494</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="13" x14ac:dyDescent="0.15">
@@ -16294,7 +16294,7 @@
     <row r="26" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="A26" s="110">
         <f t="shared" si="1"/>
-        <v>7.3174358974358977E-2</v>
+        <v>0.13471282051282052</v>
       </c>
       <c r="B26" s="124" t="s">
         <v>314</v>
@@ -16302,43 +16302,43 @@
       <c r="C26" s="107"/>
       <c r="D26" s="120">
         <f>D19-D20-D21-D22-D23-D24-D25</f>
-        <v>713450000</v>
+        <v>1313450000</v>
       </c>
       <c r="E26" s="120">
         <f t="shared" ref="E26:M26" si="6">E19-E20-E21-E22-E23-E24</f>
-        <v>11123869800</v>
+        <v>13283005800</v>
       </c>
       <c r="F26" s="120">
         <f t="shared" si="6"/>
-        <v>13286479564.056005</v>
+        <v>15639436884.504004</v>
       </c>
       <c r="G26" s="120">
         <f t="shared" si="6"/>
-        <v>15744996493.694756</v>
+        <v>18302934044.070896</v>
       </c>
       <c r="H26" s="120">
         <f t="shared" si="6"/>
-        <v>18536527637.347153</v>
+        <v>21311823373.128967</v>
       </c>
       <c r="I26" s="120">
         <f t="shared" si="6"/>
-        <v>21697723116.991997</v>
+        <v>24703326769.407661</v>
       </c>
       <c r="J26" s="120">
         <f t="shared" si="6"/>
-        <v>25233496965.235657</v>
+        <v>28478557060.639275</v>
       </c>
       <c r="K26" s="120">
         <f t="shared" si="6"/>
-        <v>29250465943.069538</v>
+        <v>32752901489.819916</v>
       </c>
       <c r="L26" s="120">
         <f t="shared" si="6"/>
-        <v>33841300225.799545</v>
+        <v>37623846557.836823</v>
       </c>
       <c r="M26" s="120">
         <f t="shared" si="6"/>
-        <v>39055690867.963867</v>
+        <v>43139978486.000443</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="13" x14ac:dyDescent="0.15">
@@ -16384,7 +16384,7 @@
     <row r="28" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="A28" s="110">
         <f t="shared" si="1"/>
-        <v>6.4172331381285974E-2</v>
+        <v>0.12571079291974752</v>
       </c>
       <c r="B28" s="124" t="s">
         <v>316</v>
@@ -16392,98 +16392,98 @@
       <c r="C28" s="107"/>
       <c r="D28" s="120">
         <f>D26-D27</f>
-        <v>625680230.96753824</v>
+        <v>1225680230.9675384</v>
       </c>
       <c r="E28" s="120">
         <f t="shared" ref="E28:M28" si="7">E26-E27</f>
-        <v>10954912994.612511</v>
+        <v>13114048994.612511</v>
       </c>
       <c r="F28" s="120">
         <f t="shared" si="7"/>
-        <v>13135076712.47501</v>
+        <v>15488034032.923008</v>
       </c>
       <c r="G28" s="120">
         <f t="shared" si="7"/>
-        <v>15611147595.920252</v>
+        <v>18169085146.296391</v>
       </c>
       <c r="H28" s="120">
         <f t="shared" si="7"/>
-        <v>18420232693.379143</v>
+        <v>21195528429.160957</v>
       </c>
       <c r="I28" s="120">
         <f t="shared" si="7"/>
-        <v>21598982126.830479</v>
+        <v>24604585779.246143</v>
       </c>
       <c r="J28" s="120">
         <f t="shared" si="7"/>
-        <v>25152309928.88063</v>
+        <v>28397370024.284248</v>
       </c>
       <c r="K28" s="120">
         <f t="shared" si="7"/>
-        <v>29186832860.521004</v>
+        <v>32689268407.271381</v>
       </c>
       <c r="L28" s="120">
         <f t="shared" si="7"/>
-        <v>33795221097.057503</v>
+        <v>37577767429.09478</v>
       </c>
       <c r="M28" s="120">
         <f t="shared" si="7"/>
-        <v>39033748425.70575</v>
+        <v>43118036043.742325</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="A29" s="110">
         <f t="shared" si="1"/>
-        <v>2.246031598345009E-2</v>
+        <v>4.3998777521911635E-2</v>
       </c>
       <c r="B29" s="122" t="s">
         <v>317</v>
       </c>
       <c r="D29" s="112">
         <f t="shared" ref="D29:M29" si="8">IF(D28&lt;0,0,D28*D5)</f>
-        <v>218988080.83863837</v>
+        <v>428988080.83863842</v>
       </c>
       <c r="E29" s="112">
         <f t="shared" si="8"/>
-        <v>3834219548.1143785</v>
+        <v>4589917148.114378</v>
       </c>
       <c r="F29" s="112">
         <f t="shared" si="8"/>
-        <v>4597276849.3662529</v>
+        <v>5420811911.5230522</v>
       </c>
       <c r="G29" s="112">
         <f t="shared" si="8"/>
-        <v>5463901658.5720882</v>
+        <v>6359179801.2037363</v>
       </c>
       <c r="H29" s="112">
         <f t="shared" si="8"/>
-        <v>6447081442.6826992</v>
+        <v>7418434950.2063351</v>
       </c>
       <c r="I29" s="112">
         <f t="shared" si="8"/>
-        <v>7559643744.390667</v>
+        <v>8611605022.7361488</v>
       </c>
       <c r="J29" s="112">
         <f t="shared" si="8"/>
-        <v>8803308475.1082211</v>
+        <v>9939079508.4994869</v>
       </c>
       <c r="K29" s="112">
         <f t="shared" si="8"/>
-        <v>10215391501.18235</v>
+        <v>11441243942.544983</v>
       </c>
       <c r="L29" s="112">
         <f t="shared" si="8"/>
-        <v>11828327383.970125</v>
+        <v>13152218600.183172</v>
       </c>
       <c r="M29" s="112">
         <f t="shared" si="8"/>
-        <v>13661811948.997011</v>
+        <v>15091312615.309813</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="A30" s="110">
         <f t="shared" si="1"/>
-        <v>4.1712015397835887E-2</v>
+        <v>8.1712015397835888E-2</v>
       </c>
       <c r="B30" s="124" t="s">
         <v>318</v>
@@ -16491,43 +16491,43 @@
       <c r="C30" s="107"/>
       <c r="D30" s="120">
         <f>D28-D29</f>
-        <v>406692150.12889987</v>
+        <v>796692150.12889993</v>
       </c>
       <c r="E30" s="120">
         <f t="shared" ref="E30:M30" si="9">E28-E29</f>
-        <v>7120693446.4981327</v>
+        <v>8524131846.4981327</v>
       </c>
       <c r="F30" s="120">
         <f t="shared" si="9"/>
-        <v>8537799863.108757</v>
+        <v>10067222121.399956</v>
       </c>
       <c r="G30" s="120">
         <f t="shared" si="9"/>
-        <v>10147245937.348164</v>
+        <v>11809905345.092655</v>
       </c>
       <c r="H30" s="120">
         <f t="shared" si="9"/>
-        <v>11973151250.696444</v>
+        <v>13777093478.954622</v>
       </c>
       <c r="I30" s="120">
         <f t="shared" si="9"/>
-        <v>14039338382.439812</v>
+        <v>15992980756.509995</v>
       </c>
       <c r="J30" s="120">
         <f t="shared" si="9"/>
-        <v>16349001453.772409</v>
+        <v>18458290515.78476</v>
       </c>
       <c r="K30" s="120">
         <f t="shared" si="9"/>
-        <v>18971441359.338654</v>
+        <v>21248024464.726398</v>
       </c>
       <c r="L30" s="120">
         <f t="shared" si="9"/>
-        <v>21966893713.087379</v>
+        <v>24425548828.911606</v>
       </c>
       <c r="M30" s="120">
         <f t="shared" si="9"/>
-        <v>25371936476.70874</v>
+        <v>28026723428.43251</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.15">
@@ -16551,43 +16551,43 @@
       <c r="C32" s="107"/>
       <c r="D32" s="120">
         <f t="shared" ref="D32:M32" si="10">D26+D22+D23</f>
-        <v>1513250000</v>
+        <v>2113250000</v>
       </c>
       <c r="E32" s="120">
         <f t="shared" si="10"/>
-        <v>11923669800</v>
+        <v>14082805800</v>
       </c>
       <c r="F32" s="120">
         <f t="shared" si="10"/>
-        <v>14086279564.056005</v>
+        <v>16439236884.504004</v>
       </c>
       <c r="G32" s="120">
         <f t="shared" si="10"/>
-        <v>16544796493.694756</v>
+        <v>19102734044.070896</v>
       </c>
       <c r="H32" s="120">
         <f t="shared" si="10"/>
-        <v>19336327637.347153</v>
+        <v>22111623373.128967</v>
       </c>
       <c r="I32" s="120">
         <f t="shared" si="10"/>
-        <v>22497523116.991997</v>
+        <v>25503126769.407661</v>
       </c>
       <c r="J32" s="120">
         <f t="shared" si="10"/>
-        <v>26033296965.235657</v>
+        <v>29278357060.639275</v>
       </c>
       <c r="K32" s="120">
         <f t="shared" si="10"/>
-        <v>30050265943.069538</v>
+        <v>33552701489.819916</v>
       </c>
       <c r="L32" s="120">
         <f t="shared" si="10"/>
-        <v>34641100225.799545</v>
+        <v>38423646557.836823</v>
       </c>
       <c r="M32" s="120">
         <f t="shared" si="10"/>
-        <v>39855490867.963867</v>
+        <v>43939778486.000443</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.15">
@@ -16692,99 +16692,99 @@
     <row r="36" spans="1:16" ht="13" x14ac:dyDescent="0.15">
       <c r="A36" s="110">
         <f t="shared" si="1"/>
-        <v>7.6923076923076927E-2</v>
+        <v>6.1538461538461542E-2</v>
       </c>
       <c r="B36" s="122" t="s">
         <v>322</v>
       </c>
       <c r="D36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!D16</f>
-        <v>750000000</v>
+        <v>600000000</v>
       </c>
       <c r="E36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!E16</f>
-        <v>2698920000</v>
+        <v>2159136000</v>
       </c>
       <c r="F36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!F16</f>
-        <v>2941196650.5599999</v>
+        <v>2352957320.448</v>
       </c>
       <c r="G36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!G16</f>
-        <v>3197421937.9701848</v>
+        <v>2557937550.3761482</v>
       </c>
       <c r="H36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!H16</f>
-        <v>3469119669.7272639</v>
+        <v>2775295735.7818108</v>
       </c>
       <c r="I36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!I16</f>
-        <v>3757004565.5195813</v>
+        <v>3005603652.4156642</v>
       </c>
       <c r="J36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!J16</f>
-        <v>4056325119.2545261</v>
+        <v>3245060095.4036207</v>
       </c>
       <c r="K36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!K16</f>
-        <v>4378044433.4379606</v>
+        <v>3502435546.7503676</v>
       </c>
       <c r="L36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!L16</f>
-        <v>4728182915.0465956</v>
+        <v>3782546332.0372748</v>
       </c>
       <c r="M36" s="112">
         <f>(Datos!$C$29/360)*'Estado de resultados'!M16</f>
-        <v>5105359522.5456924</v>
+        <v>4084287618.0365524</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="13" x14ac:dyDescent="0.15">
       <c r="A37" s="110">
         <f t="shared" si="1"/>
-        <v>2.246031598345009E-2</v>
+        <v>4.3998777521911635E-2</v>
       </c>
       <c r="B37" s="122" t="s">
         <v>323</v>
       </c>
       <c r="D37" s="112">
         <f>D29</f>
-        <v>218988080.83863837</v>
+        <v>428988080.83863842</v>
       </c>
       <c r="E37" s="112">
         <f t="shared" ref="E37:M37" si="12">E29</f>
-        <v>3834219548.1143785</v>
+        <v>4589917148.114378</v>
       </c>
       <c r="F37" s="112">
         <f t="shared" si="12"/>
-        <v>4597276849.3662529</v>
+        <v>5420811911.5230522</v>
       </c>
       <c r="G37" s="112">
         <f t="shared" si="12"/>
-        <v>5463901658.5720882</v>
+        <v>6359179801.2037363</v>
       </c>
       <c r="H37" s="112">
         <f t="shared" si="12"/>
-        <v>6447081442.6826992</v>
+        <v>7418434950.2063351</v>
       </c>
       <c r="I37" s="112">
         <f t="shared" si="12"/>
-        <v>7559643744.390667</v>
+        <v>8611605022.7361488</v>
       </c>
       <c r="J37" s="112">
         <f t="shared" si="12"/>
-        <v>8803308475.1082211</v>
+        <v>9939079508.4994869</v>
       </c>
       <c r="K37" s="112">
         <f t="shared" si="12"/>
-        <v>10215391501.18235</v>
+        <v>11441243942.544983</v>
       </c>
       <c r="L37" s="112">
         <f t="shared" si="12"/>
-        <v>11828327383.970125</v>
+        <v>13152218600.183172</v>
       </c>
       <c r="M37" s="112">
         <f t="shared" si="12"/>
-        <v>13661811948.997011</v>
+        <v>15091312615.309813</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="13" x14ac:dyDescent="0.15">
@@ -16795,43 +16795,43 @@
       <c r="C38" s="107"/>
       <c r="D38" s="120">
         <f>D35-D36-D37</f>
-        <v>-156488080.83863837</v>
+        <v>-216488080.83863842</v>
       </c>
       <c r="E38" s="120">
         <f>E35-E36-E37</f>
-        <v>-3494649548.1143785</v>
+        <v>-3710563148.114378</v>
       </c>
       <c r="F38" s="120">
         <f t="shared" ref="F38:M38" si="13">F35-F36-F37</f>
-        <v>-4097371420.9662528</v>
+        <v>-4332667153.0110521</v>
       </c>
       <c r="G38" s="120">
         <f t="shared" si="13"/>
-        <v>-4773745405.0413704</v>
+        <v>-5029539160.0789814</v>
       </c>
       <c r="H38" s="120">
         <f t="shared" si="13"/>
-        <v>-5532871174.7724819</v>
+        <v>-5810400748.3506641</v>
       </c>
       <c r="I38" s="120">
         <f t="shared" si="13"/>
-        <v>-6383407714.9464569</v>
+        <v>-6683968080.1880207</v>
       </c>
       <c r="J38" s="120">
         <f t="shared" si="13"/>
-        <v>-7324488314.407423</v>
+        <v>-7648994323.9477835</v>
       </c>
       <c r="K38" s="120">
         <f t="shared" si="13"/>
-        <v>-8385001117.956502</v>
+        <v>-8735244672.6315422</v>
       </c>
       <c r="L38" s="120">
         <f t="shared" si="13"/>
-        <v>-9588610068.1000595</v>
+        <v>-9966864701.3037872</v>
       </c>
       <c r="M38" s="120">
         <f t="shared" si="13"/>
-        <v>-10948379136.027424</v>
+        <v>-11356807897.831085</v>
       </c>
       <c r="O38" s="108" t="s">
         <v>325</v>
@@ -16848,43 +16848,43 @@
       <c r="C39" s="107"/>
       <c r="D39" s="120">
         <f>D38</f>
-        <v>-156488080.83863837</v>
+        <v>-216488080.83863842</v>
       </c>
       <c r="E39" s="120">
         <f>E38-D38</f>
-        <v>-3338161467.2757401</v>
+        <v>-3494075067.2757397</v>
       </c>
       <c r="F39" s="120">
         <f t="shared" ref="F39:M39" si="14">F38-E38</f>
-        <v>-602721872.85187435</v>
+        <v>-622104004.89667416</v>
       </c>
       <c r="G39" s="120">
         <f t="shared" si="14"/>
-        <v>-676373984.07511759</v>
+        <v>-696872007.06792927</v>
       </c>
       <c r="H39" s="120">
         <f t="shared" si="14"/>
-        <v>-759125769.73111153</v>
+        <v>-780861588.27168274</v>
       </c>
       <c r="I39" s="120">
         <f t="shared" si="14"/>
-        <v>-850536540.17397499</v>
+        <v>-873567331.83735657</v>
       </c>
       <c r="J39" s="120">
         <f t="shared" si="14"/>
-        <v>-941080599.46096611</v>
+        <v>-965026243.75976276</v>
       </c>
       <c r="K39" s="120">
         <f t="shared" si="14"/>
-        <v>-1060512803.5490789</v>
+        <v>-1086250348.6837587</v>
       </c>
       <c r="L39" s="120">
         <f t="shared" si="14"/>
-        <v>-1203608950.1435575</v>
+        <v>-1231620028.672245</v>
       </c>
       <c r="M39" s="120">
         <f t="shared" si="14"/>
-        <v>-1359769067.9273643</v>
+        <v>-1389943196.527298</v>
       </c>
       <c r="O39" s="108" t="s">
         <v>327</v>
@@ -17100,43 +17100,43 @@
       <c r="C45" s="107"/>
       <c r="D45" s="120">
         <f>D43+D38</f>
-        <v>13043711919.161362</v>
+        <v>12983711919.161362</v>
       </c>
       <c r="E45" s="120">
         <f>E43+E38</f>
-        <v>8905750451.885622</v>
+        <v>8689836851.885622</v>
       </c>
       <c r="F45" s="120">
         <f t="shared" ref="F45:L45" si="18">F43+F38</f>
-        <v>7503228579.0337467</v>
+        <v>7267932846.9889479</v>
       </c>
       <c r="G45" s="120">
         <f t="shared" si="18"/>
-        <v>6027054594.9586296</v>
+        <v>5771260839.9210186</v>
       </c>
       <c r="H45" s="120">
         <f t="shared" si="18"/>
-        <v>4468128825.2275181</v>
+        <v>4190599251.6493359</v>
       </c>
       <c r="I45" s="120">
         <f t="shared" si="18"/>
-        <v>2817792285.0535431</v>
+        <v>2517231919.8119793</v>
       </c>
       <c r="J45" s="120">
         <f t="shared" si="18"/>
-        <v>1076911685.592577</v>
+        <v>752405676.05221653</v>
       </c>
       <c r="K45" s="120">
         <f t="shared" si="18"/>
-        <v>-783401117.95650196</v>
+        <v>-1133644672.6315422</v>
       </c>
       <c r="L45" s="120">
         <f t="shared" si="18"/>
-        <v>-2786810068.1000595</v>
+        <v>-3165064701.3037872</v>
       </c>
       <c r="M45" s="120">
         <f>M43+M38</f>
-        <v>-4946379136.0274239</v>
+        <v>-5354807897.8310852</v>
       </c>
       <c r="O45" s="108" t="s">
         <v>335</v>
@@ -17223,43 +17223,43 @@
       <c r="C49" s="112"/>
       <c r="D49" s="112">
         <f>D26</f>
-        <v>713450000</v>
+        <v>1313450000</v>
       </c>
       <c r="E49" s="112">
         <f t="shared" ref="E49:M49" si="19">E26</f>
-        <v>11123869800</v>
+        <v>13283005800</v>
       </c>
       <c r="F49" s="112">
         <f t="shared" si="19"/>
-        <v>13286479564.056005</v>
+        <v>15639436884.504004</v>
       </c>
       <c r="G49" s="112">
         <f t="shared" si="19"/>
-        <v>15744996493.694756</v>
+        <v>18302934044.070896</v>
       </c>
       <c r="H49" s="112">
         <f t="shared" si="19"/>
-        <v>18536527637.347153</v>
+        <v>21311823373.128967</v>
       </c>
       <c r="I49" s="112">
         <f t="shared" si="19"/>
-        <v>21697723116.991997</v>
+        <v>24703326769.407661</v>
       </c>
       <c r="J49" s="112">
         <f t="shared" si="19"/>
-        <v>25233496965.235657</v>
+        <v>28478557060.639275</v>
       </c>
       <c r="K49" s="112">
         <f t="shared" si="19"/>
-        <v>29250465943.069538</v>
+        <v>32752901489.819916</v>
       </c>
       <c r="L49" s="112">
         <f t="shared" si="19"/>
-        <v>33841300225.799545</v>
+        <v>37623846557.836823</v>
       </c>
       <c r="M49" s="112">
         <f t="shared" si="19"/>
-        <v>39055690867.963867</v>
+        <v>43139978486.000443</v>
       </c>
       <c r="O49" s="108" t="s">
         <v>339</v>
@@ -17276,43 +17276,43 @@
       <c r="C50" s="112"/>
       <c r="D50" s="112">
         <f t="shared" ref="D50:M50" si="20">IF(D49&lt;0,0,D49*D5)</f>
-        <v>249707499.99999997</v>
+        <v>459707500</v>
       </c>
       <c r="E50" s="112">
         <f t="shared" si="20"/>
-        <v>3893354429.9999995</v>
+        <v>4649052030</v>
       </c>
       <c r="F50" s="112">
         <f t="shared" si="20"/>
-        <v>4650267847.4196014</v>
+        <v>5473802909.5764008</v>
       </c>
       <c r="G50" s="112">
         <f t="shared" si="20"/>
-        <v>5510748772.7931643</v>
+        <v>6406026915.4248133</v>
       </c>
       <c r="H50" s="112">
         <f t="shared" si="20"/>
-        <v>6487784673.0715027</v>
+        <v>7459138180.5951385</v>
       </c>
       <c r="I50" s="112">
         <f t="shared" si="20"/>
-        <v>7594203090.9471979</v>
+        <v>8646164369.2926807</v>
       </c>
       <c r="J50" s="112">
         <f t="shared" si="20"/>
-        <v>8831723937.8324795</v>
+        <v>9967494971.2237453</v>
       </c>
       <c r="K50" s="112">
         <f t="shared" si="20"/>
-        <v>10237663080.074337</v>
+        <v>11463515521.43697</v>
       </c>
       <c r="L50" s="112">
         <f t="shared" si="20"/>
-        <v>11844455079.02984</v>
+        <v>13168346295.242887</v>
       </c>
       <c r="M50" s="112">
         <f t="shared" si="20"/>
-        <v>13669491803.787354</v>
+        <v>15098992470.100153</v>
       </c>
     </row>
     <row r="51" spans="2:16" s="107" customFormat="1" ht="13" x14ac:dyDescent="0.15">
@@ -17322,43 +17322,43 @@
       <c r="C51" s="120"/>
       <c r="D51" s="120">
         <f>D49-D50</f>
-        <v>463742500</v>
+        <v>853742500</v>
       </c>
       <c r="E51" s="120">
         <f t="shared" ref="E51:M51" si="21">E49-E50</f>
-        <v>7230515370</v>
+        <v>8633953770</v>
       </c>
       <c r="F51" s="120">
         <f t="shared" si="21"/>
-        <v>8636211716.636404</v>
+        <v>10165633974.927603</v>
       </c>
       <c r="G51" s="120">
         <f t="shared" si="21"/>
-        <v>10234247720.901592</v>
+        <v>11896907128.646084</v>
       </c>
       <c r="H51" s="120">
         <f t="shared" si="21"/>
-        <v>12048742964.27565</v>
+        <v>13852685192.533829</v>
       </c>
       <c r="I51" s="120">
         <f t="shared" si="21"/>
-        <v>14103520026.0448</v>
+        <v>16057162400.114981</v>
       </c>
       <c r="J51" s="120">
         <f t="shared" si="21"/>
-        <v>16401773027.403177</v>
+        <v>18511062089.415527</v>
       </c>
       <c r="K51" s="120">
         <f t="shared" si="21"/>
-        <v>19012802862.995201</v>
+        <v>21289385968.382946</v>
       </c>
       <c r="L51" s="120">
         <f t="shared" si="21"/>
-        <v>21996845146.769707</v>
+        <v>24455500262.593933</v>
       </c>
       <c r="M51" s="120">
         <f t="shared" si="21"/>
-        <v>25386199064.176514</v>
+        <v>28040986015.900291</v>
       </c>
     </row>
     <row r="52" spans="2:16" ht="13" x14ac:dyDescent="0.15">
@@ -17424,43 +17424,43 @@
       <c r="C54" s="120"/>
       <c r="D54" s="120">
         <f t="shared" ref="D54:M54" si="22">D51+D52+D53</f>
-        <v>1263542500</v>
+        <v>1653542500</v>
       </c>
       <c r="E54" s="120">
         <f t="shared" si="22"/>
-        <v>8030315370</v>
+        <v>9433753770</v>
       </c>
       <c r="F54" s="120">
         <f t="shared" si="22"/>
-        <v>9436011716.636404</v>
+        <v>10965433974.927603</v>
       </c>
       <c r="G54" s="120">
         <f t="shared" si="22"/>
-        <v>11034047720.901592</v>
+        <v>12696707128.646084</v>
       </c>
       <c r="H54" s="120">
         <f t="shared" si="22"/>
-        <v>12848542964.27565</v>
+        <v>14652485192.533829</v>
       </c>
       <c r="I54" s="120">
         <f t="shared" si="22"/>
-        <v>14903320026.0448</v>
+        <v>16856962400.114981</v>
       </c>
       <c r="J54" s="120">
         <f t="shared" si="22"/>
-        <v>17201573027.403175</v>
+        <v>19310862089.415527</v>
       </c>
       <c r="K54" s="120">
         <f t="shared" si="22"/>
-        <v>19812602862.995201</v>
+        <v>22089185968.382946</v>
       </c>
       <c r="L54" s="120">
         <f t="shared" si="22"/>
-        <v>22796645146.769707</v>
+        <v>25255300262.593933</v>
       </c>
       <c r="M54" s="120">
         <f t="shared" si="22"/>
-        <v>26185999064.176514</v>
+        <v>28840786015.900291</v>
       </c>
     </row>
     <row r="55" spans="2:16" x14ac:dyDescent="0.15">
@@ -17539,43 +17539,43 @@
       <c r="C58" s="107"/>
       <c r="D58" s="137">
         <f t="shared" ref="D58:M58" si="23">D32</f>
-        <v>1513250000</v>
+        <v>2113250000</v>
       </c>
       <c r="E58" s="137">
         <f t="shared" si="23"/>
-        <v>11923669800</v>
+        <v>14082805800</v>
       </c>
       <c r="F58" s="137">
         <f t="shared" si="23"/>
-        <v>14086279564.056005</v>
+        <v>16439236884.504004</v>
       </c>
       <c r="G58" s="137">
         <f t="shared" si="23"/>
-        <v>16544796493.694756</v>
+        <v>19102734044.070896</v>
       </c>
       <c r="H58" s="137">
         <f t="shared" si="23"/>
-        <v>19336327637.347153</v>
+        <v>22111623373.128967</v>
       </c>
       <c r="I58" s="137">
         <f t="shared" si="23"/>
-        <v>22497523116.991997</v>
+        <v>25503126769.407661</v>
       </c>
       <c r="J58" s="137">
         <f t="shared" si="23"/>
-        <v>26033296965.235657</v>
+        <v>29278357060.639275</v>
       </c>
       <c r="K58" s="137">
         <f t="shared" si="23"/>
-        <v>30050265943.069538</v>
+        <v>33552701489.819916</v>
       </c>
       <c r="L58" s="137">
         <f t="shared" si="23"/>
-        <v>34641100225.799545</v>
+        <v>38423646557.836823</v>
       </c>
       <c r="M58" s="137">
         <f t="shared" si="23"/>
-        <v>39855490867.963867</v>
+        <v>43939778486.000443</v>
       </c>
       <c r="N58" s="107"/>
     </row>
@@ -17586,43 +17586,43 @@
       <c r="C59" s="107"/>
       <c r="D59" s="137">
         <f t="shared" ref="D59:M59" si="24">D50</f>
-        <v>249707499.99999997</v>
+        <v>459707500</v>
       </c>
       <c r="E59" s="137">
         <f t="shared" si="24"/>
-        <v>3893354429.9999995</v>
+        <v>4649052030</v>
       </c>
       <c r="F59" s="137">
         <f t="shared" si="24"/>
-        <v>4650267847.4196014</v>
+        <v>5473802909.5764008</v>
       </c>
       <c r="G59" s="137">
         <f t="shared" si="24"/>
-        <v>5510748772.7931643</v>
+        <v>6406026915.4248133</v>
       </c>
       <c r="H59" s="137">
         <f t="shared" si="24"/>
-        <v>6487784673.0715027</v>
+        <v>7459138180.5951385</v>
       </c>
       <c r="I59" s="137">
         <f t="shared" si="24"/>
-        <v>7594203090.9471979</v>
+        <v>8646164369.2926807</v>
       </c>
       <c r="J59" s="137">
         <f t="shared" si="24"/>
-        <v>8831723937.8324795</v>
+        <v>9967494971.2237453</v>
       </c>
       <c r="K59" s="137">
         <f t="shared" si="24"/>
-        <v>10237663080.074337</v>
+        <v>11463515521.43697</v>
       </c>
       <c r="L59" s="137">
         <f t="shared" si="24"/>
-        <v>11844455079.02984</v>
+        <v>13168346295.242887</v>
       </c>
       <c r="M59" s="137">
         <f t="shared" si="24"/>
-        <v>13669491803.787354</v>
+        <v>15098992470.100153</v>
       </c>
       <c r="N59" s="107"/>
     </row>
@@ -17632,43 +17632,43 @@
       </c>
       <c r="D60" s="138">
         <f>D58-D59</f>
-        <v>1263542500</v>
+        <v>1653542500</v>
       </c>
       <c r="E60" s="138">
         <f t="shared" ref="E60:M60" si="25">E58-E59</f>
-        <v>8030315370</v>
+        <v>9433753770</v>
       </c>
       <c r="F60" s="138">
         <f t="shared" si="25"/>
-        <v>9436011716.636404</v>
+        <v>10965433974.927603</v>
       </c>
       <c r="G60" s="138">
         <f t="shared" si="25"/>
-        <v>11034047720.901592</v>
+        <v>12696707128.646084</v>
       </c>
       <c r="H60" s="138">
         <f t="shared" si="25"/>
-        <v>12848542964.27565</v>
+        <v>14652485192.533829</v>
       </c>
       <c r="I60" s="138">
         <f t="shared" si="25"/>
-        <v>14903320026.0448</v>
+        <v>16856962400.114981</v>
       </c>
       <c r="J60" s="138">
         <f t="shared" si="25"/>
-        <v>17201573027.403175</v>
+        <v>19310862089.415527</v>
       </c>
       <c r="K60" s="138">
         <f t="shared" si="25"/>
-        <v>19812602862.995201</v>
+        <v>22089185968.382946</v>
       </c>
       <c r="L60" s="138">
         <f t="shared" si="25"/>
-        <v>22796645146.769707</v>
+        <v>25255300262.593933</v>
       </c>
       <c r="M60" s="138">
         <f t="shared" si="25"/>
-        <v>26185999064.176514</v>
+        <v>28840786015.900291</v>
       </c>
     </row>
     <row r="61" spans="2:16" ht="13" x14ac:dyDescent="0.15">
@@ -17678,43 +17678,43 @@
       <c r="C61" s="112"/>
       <c r="D61" s="112">
         <f t="shared" ref="D61:M61" si="26">-D39</f>
-        <v>156488080.83863837</v>
+        <v>216488080.83863842</v>
       </c>
       <c r="E61" s="112">
         <f t="shared" si="26"/>
-        <v>3338161467.2757401</v>
+        <v>3494075067.2757397</v>
       </c>
       <c r="F61" s="112">
         <f t="shared" si="26"/>
-        <v>602721872.85187435</v>
+        <v>622104004.89667416</v>
       </c>
       <c r="G61" s="112">
         <f t="shared" si="26"/>
-        <v>676373984.07511759</v>
+        <v>696872007.06792927</v>
       </c>
       <c r="H61" s="112">
         <f t="shared" si="26"/>
-        <v>759125769.73111153</v>
+        <v>780861588.27168274</v>
       </c>
       <c r="I61" s="112">
         <f t="shared" si="26"/>
-        <v>850536540.17397499</v>
+        <v>873567331.83735657</v>
       </c>
       <c r="J61" s="112">
         <f t="shared" si="26"/>
-        <v>941080599.46096611</v>
+        <v>965026243.75976276</v>
       </c>
       <c r="K61" s="112">
         <f t="shared" si="26"/>
-        <v>1060512803.5490789</v>
+        <v>1086250348.6837587</v>
       </c>
       <c r="L61" s="112">
         <f t="shared" si="26"/>
-        <v>1203608950.1435575</v>
+        <v>1231620028.672245</v>
       </c>
       <c r="M61" s="112">
         <f t="shared" si="26"/>
-        <v>1359769067.9273643</v>
+        <v>1389943196.527298</v>
       </c>
     </row>
     <row r="62" spans="2:16" s="107" customFormat="1" ht="13" x14ac:dyDescent="0.15">
@@ -17724,43 +17724,43 @@
       <c r="C62" s="120"/>
       <c r="D62" s="120">
         <f>D60+D61</f>
-        <v>1420030580.8386383</v>
+        <v>1870030580.8386383</v>
       </c>
       <c r="E62" s="120">
         <f>E54+E61</f>
-        <v>11368476837.27574</v>
+        <v>12927828837.27574</v>
       </c>
       <c r="F62" s="120">
         <f>F54+F61</f>
-        <v>10038733589.488277</v>
+        <v>11587537979.824276</v>
       </c>
       <c r="G62" s="120">
         <f>G54+G61</f>
-        <v>11710421704.976709</v>
+        <v>13393579135.714012</v>
       </c>
       <c r="H62" s="120">
         <f t="shared" ref="H62:M62" si="27">H54+H61</f>
-        <v>13607668734.006762</v>
+        <v>15433346780.805511</v>
       </c>
       <c r="I62" s="120">
         <f t="shared" si="27"/>
-        <v>15753856566.218775</v>
+        <v>17730529731.952339</v>
       </c>
       <c r="J62" s="120">
         <f t="shared" si="27"/>
-        <v>18142653626.864143</v>
+        <v>20275888333.175289</v>
       </c>
       <c r="K62" s="120">
         <f t="shared" si="27"/>
-        <v>20873115666.544281</v>
+        <v>23175436317.066704</v>
       </c>
       <c r="L62" s="120">
         <f t="shared" si="27"/>
-        <v>24000254096.913265</v>
+        <v>26486920291.266178</v>
       </c>
       <c r="M62" s="120">
         <f t="shared" si="27"/>
-        <v>27545768132.103878</v>
+        <v>30230729212.427589</v>
       </c>
     </row>
     <row r="63" spans="2:16" ht="13" x14ac:dyDescent="0.15">
@@ -17813,43 +17813,43 @@
       </c>
       <c r="D64" s="120">
         <f>D62+D63</f>
-        <v>1420030580.8386383</v>
+        <v>1870030580.8386383</v>
       </c>
       <c r="E64" s="120">
         <f t="shared" ref="E64:L64" si="28">E62+E63</f>
-        <v>11368476837.27574</v>
+        <v>12927828837.27574</v>
       </c>
       <c r="F64" s="120">
         <f>F62+F63</f>
-        <v>10038733589.488277</v>
+        <v>11587537979.824276</v>
       </c>
       <c r="G64" s="120">
         <f>G62+G63</f>
-        <v>11710421704.976709</v>
+        <v>13393579135.714012</v>
       </c>
       <c r="H64" s="120">
         <f>H62+H63</f>
-        <v>3807668734.0067616</v>
+        <v>5633346780.8055115</v>
       </c>
       <c r="I64" s="120">
         <f t="shared" si="28"/>
-        <v>15753856566.218775</v>
+        <v>17730529731.952339</v>
       </c>
       <c r="J64" s="120">
         <f t="shared" si="28"/>
-        <v>18142653626.864143</v>
+        <v>20275888333.175289</v>
       </c>
       <c r="K64" s="120">
         <f t="shared" si="28"/>
-        <v>20873115666.544281</v>
+        <v>23175436317.066704</v>
       </c>
       <c r="L64" s="120">
         <f t="shared" si="28"/>
-        <v>24000254096.913265</v>
+        <v>26486920291.266178</v>
       </c>
       <c r="M64" s="120">
         <f>M62+M63</f>
-        <v>27545768132.103878</v>
+        <v>30230729212.427589</v>
       </c>
       <c r="N64" s="121">
         <f>P49</f>
@@ -17916,43 +17916,43 @@
       </c>
       <c r="D66" s="112">
         <f t="shared" ref="D66:N66" si="29">D64*D65</f>
-        <v>1179537260.6334753</v>
+        <v>1553326230.0031278</v>
       </c>
       <c r="E66" s="112">
         <f t="shared" si="29"/>
-        <v>7843866903.4200974</v>
+        <v>8919767370.884388</v>
       </c>
       <c r="F66" s="112">
         <f t="shared" si="29"/>
-        <v>5753350477.9872265</v>
+        <v>6640993764.863471</v>
       </c>
       <c r="G66" s="112">
         <f t="shared" si="29"/>
-        <v>5574788608.3949623</v>
+        <v>6376061791.1550627</v>
       </c>
       <c r="H66" s="112">
         <f t="shared" si="29"/>
-        <v>1505667216.0945742</v>
+        <v>2227595454.6669092</v>
       </c>
       <c r="I66" s="112">
         <f t="shared" si="29"/>
-        <v>5174527397.9237785</v>
+        <v>5823787432.1151438</v>
       </c>
       <c r="J66" s="112">
         <f t="shared" si="29"/>
-        <v>4949924562.4919052</v>
+        <v>5531942556.5241737</v>
       </c>
       <c r="K66" s="112">
         <f t="shared" si="29"/>
-        <v>4730412548.2766924</v>
+        <v>5252180676.6852341</v>
       </c>
       <c r="L66" s="112">
         <f t="shared" si="29"/>
-        <v>4517951300.7960358</v>
+        <v>4986056210.1047745</v>
       </c>
       <c r="M66" s="112">
         <f t="shared" si="29"/>
-        <v>4307195260.8930149</v>
+        <v>4727029319.8087358</v>
       </c>
       <c r="N66" s="112">
         <f t="shared" si="29"/>
@@ -18007,49 +18007,49 @@
       <c r="N67" s="112"/>
     </row>
     <row r="68" spans="2:14" ht="13" x14ac:dyDescent="0.15">
-      <c r="B68" s="167" t="s">
+      <c r="B68" s="156" t="s">
         <v>375</v>
       </c>
       <c r="C68" s="137"/>
       <c r="D68" s="112">
         <f>D64+D67-D27*(1-D5)</f>
-        <v>9762980230.9675388</v>
+        <v>10212980230.967539</v>
       </c>
       <c r="E68" s="112">
         <f t="shared" ref="E68:M68" si="31">E64+E67-E27*(1-E5)</f>
-        <v>10418654913.773872</v>
+        <v>11978006913.773872</v>
       </c>
       <c r="F68" s="112">
         <f t="shared" si="31"/>
-        <v>9100321735.9606304</v>
+        <v>10649126126.296629</v>
       </c>
       <c r="G68" s="112">
         <f t="shared" si="31"/>
-        <v>10783419921.423283</v>
+        <v>12466577352.160585</v>
       </c>
       <c r="H68" s="112">
         <f t="shared" si="31"/>
-        <v>2892077020.4275541</v>
+        <v>4717755067.2263041</v>
       </c>
       <c r="I68" s="112">
         <f t="shared" si="31"/>
-        <v>14849674922.613787</v>
+        <v>16826348088.347351</v>
       </c>
       <c r="J68" s="112">
         <f t="shared" si="31"/>
-        <v>17249882053.233376</v>
+        <v>19383116759.544521</v>
       </c>
       <c r="K68" s="112">
         <f t="shared" si="31"/>
-        <v>19991754162.887733</v>
+        <v>22294074813.410156</v>
       </c>
       <c r="L68" s="112">
         <f t="shared" si="31"/>
-        <v>23130302663.230938</v>
+        <v>25616968857.583851</v>
       </c>
       <c r="M68" s="112">
         <f t="shared" si="31"/>
-        <v>25851505544.636105</v>
+        <v>28536466624.959816</v>
       </c>
       <c r="N68" s="112"/>
     </row>
@@ -18087,7 +18087,7 @@
       </c>
       <c r="C71" s="141">
         <f>NPV(WACC!B18,'Estado de resultados'!D64:N64)+'Estado de resultados'!C64</f>
-        <v>31891803211.901283</v>
+        <v>38393322481.800545</v>
       </c>
       <c r="D71" s="112"/>
       <c r="E71" s="112"/>
@@ -18107,7 +18107,7 @@
       </c>
       <c r="C72" s="143">
         <f>MIRR(C64:N64,WACC!B18,WACC!B18)</f>
-        <v>0.34109457050803416</v>
+        <v>0.35734543802520369</v>
       </c>
       <c r="D72" s="112"/>
       <c r="E72" s="112"/>
@@ -18125,9 +18125,9 @@
       <c r="B73" s="142" t="s">
         <v>351</v>
       </c>
-      <c r="C73" s="166">
+      <c r="C73" s="155">
         <f>2+ABS(SUM(C66:E66))/F66</f>
-        <v>2.8649909048627014</v>
+        <v>2.5310811188790496</v>
       </c>
       <c r="D73" s="120"/>
       <c r="E73" s="120"/>
@@ -18159,7 +18159,7 @@
       </c>
       <c r="C76" s="148">
         <f>ABS(SUM(D66:N66)/C64)</f>
-        <v>3.2779859437072347</v>
+        <v>3.742380177271468</v>
       </c>
       <c r="D76" s="120"/>
       <c r="E76" s="120"/>
@@ -18177,44 +18177,44 @@
         <v>355</v>
       </c>
       <c r="D79" s="116">
-        <f>D51/D45</f>
-        <v>3.5552954778061065E-2</v>
+        <f t="shared" ref="D79:M79" si="32">D51/D45</f>
+        <v>6.5754886223256911E-2</v>
       </c>
       <c r="E79" s="116">
-        <f>E51/E45</f>
-        <v>0.81189287854670089</v>
+        <f t="shared" si="32"/>
+        <v>0.9935691448714028</v>
       </c>
       <c r="F79" s="116">
-        <f>F51/F45</f>
-        <v>1.1509994165403077</v>
+        <f t="shared" si="32"/>
+        <v>1.398696739354045</v>
       </c>
       <c r="G79" s="116">
-        <f>G51/G45</f>
-        <v>1.6980512719201346</v>
+        <f t="shared" si="32"/>
+        <v>2.0614052039292154</v>
       </c>
       <c r="H79" s="116">
-        <f>H51/H45</f>
-        <v>2.6965970399616053</v>
+        <f t="shared" si="32"/>
+        <v>3.305657344133226</v>
       </c>
       <c r="I79" s="116">
-        <f>I51/I45</f>
-        <v>5.0051666692588759</v>
+        <f t="shared" si="32"/>
+        <v>6.3788967054391819</v>
       </c>
       <c r="J79" s="116">
-        <f>J51/J45</f>
-        <v>15.230378912991371</v>
+        <f t="shared" si="32"/>
+        <v>24.60250191963048</v>
       </c>
       <c r="K79" s="116">
-        <f>K51/K45</f>
-        <v>-24.269563097624886</v>
+        <f t="shared" si="32"/>
+        <v>-18.779593361439836</v>
       </c>
       <c r="L79" s="116">
-        <f>L51/L45</f>
-        <v>-7.8931985349709581</v>
+        <f t="shared" si="32"/>
+        <v>-7.7266983681312933</v>
       </c>
       <c r="M79" s="116">
-        <f>M51/M45</f>
-        <v>-5.1322792624758007</v>
+        <f t="shared" si="32"/>
+        <v>-5.2365998091655221</v>
       </c>
     </row>
     <row r="80" spans="2:14" ht="13" x14ac:dyDescent="0.15">
@@ -18222,44 +18222,44 @@
         <v>356</v>
       </c>
       <c r="D80" s="116">
-        <f>D19/D15</f>
-        <v>0.60653846153846158</v>
+        <f t="shared" ref="D80:M80" si="33">D19/D15</f>
+        <v>0.66807692307692312</v>
       </c>
       <c r="E80" s="116">
-        <f>E19/E15</f>
-        <v>0.64021044992743104</v>
+        <f t="shared" si="33"/>
+        <v>0.69942670537010154</v>
       </c>
       <c r="F80" s="116">
-        <f>F19/F15</f>
-        <v>0.65187624941807931</v>
+        <f t="shared" si="33"/>
+        <v>0.70885792918366786</v>
       </c>
       <c r="G80" s="116">
-        <f>G19/G15</f>
-        <v>0.66309252966181187</v>
+        <f t="shared" si="33"/>
+        <v>0.7179239573607743</v>
       </c>
       <c r="H80" s="116">
-        <f>H19/H15</f>
-        <v>0.6738767800867127</v>
+        <f t="shared" si="33"/>
+        <v>0.72663909730646925</v>
       </c>
       <c r="I80" s="116">
-        <f>I19/I15</f>
-        <v>0.68424580034409155</v>
+        <f t="shared" si="33"/>
+        <v>0.7350170867253667</v>
       </c>
       <c r="J80" s="116">
-        <f>J19/J15</f>
-        <v>0.69421572802449438</v>
+        <f t="shared" si="33"/>
+        <v>0.74307111680647608</v>
       </c>
       <c r="K80" s="116">
-        <f>K19/K15</f>
-        <v>0.70380206523235489</v>
+        <f t="shared" si="33"/>
+        <v>0.75081385443765813</v>
       </c>
       <c r="L80" s="116">
-        <f>L19/L15</f>
-        <v>0.71301970406775894</v>
+        <f t="shared" si="33"/>
+        <v>0.75825746349172995</v>
       </c>
       <c r="M80" s="116">
-        <f>M19/M15</f>
-        <v>0.72188295106166223</v>
+        <f t="shared" si="33"/>
+        <v>0.76541362522435141</v>
       </c>
     </row>
     <row r="81" spans="2:13" ht="13" x14ac:dyDescent="0.15">
@@ -18267,44 +18267,44 @@
         <v>357</v>
       </c>
       <c r="D81" s="116">
-        <f>D26/D15</f>
-        <v>7.3174358974358977E-2</v>
+        <f t="shared" ref="D81:M81" si="34">D26/D15</f>
+        <v>0.13471282051282052</v>
       </c>
       <c r="E81" s="116">
-        <f>E26/E15</f>
-        <v>0.30508217897705769</v>
+        <f t="shared" si="34"/>
+        <v>0.3642984344197282</v>
       </c>
       <c r="F81" s="116">
-        <f>F26/F15</f>
-        <v>0.32175930993381924</v>
+        <f t="shared" si="34"/>
+        <v>0.37874098969940778</v>
       </c>
       <c r="G81" s="116">
-        <f>G26/G15</f>
-        <v>0.33750653401897623</v>
+        <f t="shared" si="34"/>
+        <v>0.39233796171793872</v>
       </c>
       <c r="H81" s="116">
-        <f>H26/H15</f>
-        <v>0.35240574139353087</v>
+        <f t="shared" si="34"/>
+        <v>0.40516805861328742</v>
       </c>
       <c r="I81" s="116">
-        <f>I26/I15</f>
-        <v>0.36652248319868075</v>
+        <f t="shared" si="34"/>
+        <v>0.4172937695799559</v>
       </c>
       <c r="J81" s="116">
-        <f>J26/J15</f>
-        <v>0.37989814312274206</v>
+        <f t="shared" si="34"/>
+        <v>0.42875353190472371</v>
       </c>
       <c r="K81" s="116">
-        <f>K26/K15</f>
-        <v>0.39261728609063085</v>
+        <f t="shared" si="34"/>
+        <v>0.43962907529593415</v>
       </c>
       <c r="L81" s="116">
-        <f>L26/L15</f>
-        <v>0.40472857800648554</v>
+        <f t="shared" si="34"/>
+        <v>0.4499663374304565</v>
       </c>
       <c r="M81" s="116">
-        <f>M26/M15</f>
-        <v>0.4162587732225741</v>
+        <f t="shared" si="34"/>
+        <v>0.45978944738526339</v>
       </c>
     </row>
     <row r="82" spans="2:13" ht="13" x14ac:dyDescent="0.15">
@@ -18312,44 +18312,44 @@
         <v>358</v>
       </c>
       <c r="D82" s="116">
-        <f>D32/D15</f>
-        <v>0.15520512820512822</v>
+        <f t="shared" ref="D82:M82" si="35">D32/D15</f>
+        <v>0.21674358974358973</v>
       </c>
       <c r="E82" s="116">
-        <f>E32/E15</f>
-        <v>0.32701741654571842</v>
+        <f t="shared" si="35"/>
+        <v>0.38623367198838898</v>
       </c>
       <c r="F82" s="116">
-        <f>F32/F15</f>
-        <v>0.34112810471835048</v>
+        <f t="shared" si="35"/>
+        <v>0.39810978448393902</v>
       </c>
       <c r="G82" s="116">
-        <f>G32/G15</f>
-        <v>0.35465088371867143</v>
+        <f t="shared" si="35"/>
+        <v>0.40948231141763392</v>
       </c>
       <c r="H82" s="116">
-        <f>H32/H15</f>
-        <v>0.36761107636676876</v>
+        <f t="shared" si="35"/>
+        <v>0.42037339358652531</v>
       </c>
       <c r="I82" s="116">
-        <f>I32/I15</f>
-        <v>0.3800328723064087</v>
+        <f t="shared" si="35"/>
+        <v>0.43080415868768379</v>
       </c>
       <c r="J82" s="116">
-        <f>J32/J15</f>
-        <v>0.39193938081913327</v>
+        <f t="shared" si="35"/>
+        <v>0.44079476960111491</v>
       </c>
       <c r="K82" s="116">
-        <f>K32/K15</f>
-        <v>0.40335268107635375</v>
+        <f t="shared" si="35"/>
+        <v>0.45036447028165705</v>
       </c>
       <c r="L82" s="116">
-        <f>L32/L15</f>
-        <v>0.4142938699583239</v>
+        <f t="shared" si="35"/>
+        <v>0.45953162938229491</v>
       </c>
       <c r="M82" s="116">
-        <f>M32/M15</f>
-        <v>0.42478310756219528</v>
+        <f t="shared" si="35"/>
+        <v>0.46831378172488458</v>
       </c>
     </row>
     <row r="83" spans="2:13" ht="13" x14ac:dyDescent="0.15">
@@ -18357,44 +18357,44 @@
         <v>359</v>
       </c>
       <c r="D83" s="116">
-        <f>D38/D15</f>
-        <v>-1.6050059573193678E-2</v>
+        <f t="shared" ref="D83:M83" si="36">D38/D15</f>
+        <v>-2.2203905727039838E-2</v>
       </c>
       <c r="E83" s="116">
-        <f>E38/E15</f>
-        <v>-9.5843921051640191E-2</v>
+        <f t="shared" si="36"/>
+        <v>-0.10176554659590724</v>
       </c>
       <c r="F83" s="116">
-        <f>F38/F15</f>
-        <v>-9.9226239320703222E-2</v>
+        <f t="shared" si="36"/>
+        <v>-0.10492440729726207</v>
       </c>
       <c r="G83" s="116">
-        <f>G38/G15</f>
-        <v>-0.10232903300993026</v>
+        <f t="shared" si="36"/>
+        <v>-0.10781217577982644</v>
       </c>
       <c r="H83" s="116">
-        <f>H38/H15</f>
-        <v>-0.10518774640683672</v>
+        <f t="shared" si="36"/>
+        <v>-0.11046397812881238</v>
       </c>
       <c r="I83" s="116">
-        <f>I38/I15</f>
-        <v>-0.10782986004275938</v>
+        <f t="shared" si="36"/>
+        <v>-0.11290698868088685</v>
       </c>
       <c r="J83" s="116">
-        <f>J38/J15</f>
-        <v>-0.11027244911005209</v>
+        <f t="shared" si="36"/>
+        <v>-0.11515798798825023</v>
       </c>
       <c r="K83" s="116">
-        <f>K38/K15</f>
-        <v>-0.11254851082394469</v>
+        <f t="shared" si="36"/>
+        <v>-0.11724968974447506</v>
       </c>
       <c r="L83" s="116">
-        <f>L38/L15</f>
-        <v>-0.11467598738898983</v>
+        <f t="shared" si="36"/>
+        <v>-0.11919976333138693</v>
       </c>
       <c r="M83" s="116">
-        <f>M38/M15</f>
-        <v>-0.11668872747240676</v>
+        <f t="shared" si="36"/>
+        <v>-0.12104179488867572</v>
       </c>
     </row>
     <row r="85" spans="2:13" ht="13" x14ac:dyDescent="0.15">
@@ -18403,43 +18403,43 @@
       </c>
       <c r="D85" s="118">
         <f>D82/D83</f>
-        <v>-9.6700655531738402</v>
+        <v>-9.7615073855965875</v>
       </c>
       <c r="E85" s="118">
-        <f t="shared" ref="E85:M85" si="32">E82/E83</f>
-        <v>-3.411978693667209</v>
+        <f t="shared" ref="E85:M85" si="37">E82/E83</f>
+        <v>-3.7953284280194919</v>
       </c>
       <c r="F85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.4378820265052132</v>
+        <f t="shared" si="37"/>
+        <v>-3.794253355713999</v>
       </c>
       <c r="G85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.4657894566858189</v>
+        <f t="shared" si="37"/>
+        <v>-3.7981082234522097</v>
       </c>
       <c r="H85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.4948089385331271</v>
+        <f t="shared" si="37"/>
+        <v>-3.8055246670215572</v>
       </c>
       <c r="I85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.5243750864158465</v>
+        <f t="shared" si="37"/>
+        <v>-3.8155668105300493</v>
       </c>
       <c r="J85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.554281998652058</v>
+        <f t="shared" si="37"/>
+        <v>-3.827739415229189</v>
       </c>
       <c r="K85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.5838117992276488</v>
+        <f t="shared" si="37"/>
+        <v>-3.8410717440971203</v>
       </c>
       <c r="L85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.612734273244206</v>
+        <f t="shared" si="37"/>
+        <v>-3.8551387732604159</v>
       </c>
       <c r="M85" s="118">
-        <f t="shared" si="32"/>
-        <v>-3.6403097091160173</v>
+        <f t="shared" si="37"/>
+        <v>-3.8690254234547745</v>
       </c>
     </row>
     <row r="86" spans="2:13" ht="13" x14ac:dyDescent="0.15">
@@ -18448,43 +18448,43 @@
       </c>
       <c r="D86" s="119">
         <f>(D79-WACC!$B$18)*'Estado de resultados'!D45</f>
-        <v>-2195711924.9955101</v>
+        <v>-1793478653.7849333</v>
       </c>
       <c r="E86" s="119">
         <f>(E79-WACC!$B$18)*'Estado de resultados'!E45</f>
-        <v>5414741026.4728117</v>
+        <v>6862201586.9203444</v>
       </c>
       <c r="F86" s="119">
         <f>(F79-WACC!$B$18)*'Estado de resultados'!F45</f>
-        <v>7106394547.2652617</v>
+        <v>8683790747.3030453</v>
       </c>
       <c r="G86" s="119">
         <f>(G79-WACC!$B$18)*'Estado de resultados'!G45</f>
-        <v>9005404496.5502529</v>
+        <v>10720217143.950525</v>
       </c>
       <c r="H86" s="119">
         <f>(H79-WACC!$B$18)*'Estado de resultados'!H45</f>
-        <v>11137745768.895601</v>
+        <v>12998272906.196072</v>
       </c>
       <c r="I86" s="119">
         <f>(I79-WACC!$B$18)*'Estado de resultados'!I45</f>
-        <v>13529006405.409296</v>
+        <v>15543929387.198647</v>
       </c>
       <c r="J86" s="119">
         <f>(J79-WACC!$B$18)*'Estado de resultados'!J45</f>
-        <v>16182203815.408293</v>
+        <v>18357655711.156792</v>
       </c>
       <c r="K86" s="119">
         <f>(K79-WACC!$B$18)*'Estado de resultados'!K45</f>
-        <v>19172528835.372379</v>
+        <v>21520522347.328396</v>
       </c>
       <c r="L86" s="119">
         <f>(L79-WACC!$B$18)*'Estado de resultados'!L45</f>
-        <v>22565041869.693596</v>
+        <v>25100818510.761791</v>
       </c>
       <c r="M86" s="119">
         <f>(M79-WACC!$B$18)*'Estado de resultados'!M45</f>
-        <v>26394705688.86586</v>
+        <v>29132766304.14537</v>
       </c>
     </row>
     <row r="88" spans="2:13" ht="26" x14ac:dyDescent="0.15">
@@ -18492,44 +18492,44 @@
         <v>362</v>
       </c>
       <c r="D88" s="118">
-        <f>D26/D27</f>
-        <v>8.1286530415287981</v>
+        <f t="shared" ref="D88:M88" si="38">D26/D27</f>
+        <v>14.96471979451398</v>
       </c>
       <c r="E88" s="118">
-        <f>E26/E27</f>
-        <v>65.838542427979178</v>
+        <f t="shared" si="38"/>
+        <v>78.617761323886896</v>
       </c>
       <c r="F88" s="118">
-        <f>F26/F27</f>
-        <v>87.755807934357804</v>
+        <f t="shared" si="38"/>
+        <v>103.29684494837487</v>
       </c>
       <c r="G88" s="118">
-        <f>G26/G27</f>
-        <v>117.63261973378687</v>
+        <f t="shared" si="38"/>
+        <v>136.743255629239</v>
       </c>
       <c r="H88" s="118">
-        <f>H26/H27</f>
-        <v>159.3923777326539</v>
+        <f t="shared" si="38"/>
+        <v>183.25666315287984</v>
       </c>
       <c r="I88" s="118">
-        <f>I26/I27</f>
-        <v>219.7438275785882</v>
+        <f t="shared" si="38"/>
+        <v>250.18309750589123</v>
       </c>
       <c r="J88" s="118">
-        <f>J26/J27</f>
-        <v>310.80697237045035</v>
+        <f t="shared" si="38"/>
+        <v>350.77714791932891</v>
       </c>
       <c r="K88" s="118">
-        <f>K26/K27</f>
-        <v>459.6738798683748</v>
+        <f t="shared" si="38"/>
+        <v>514.71499066288914</v>
       </c>
       <c r="L88" s="118">
-        <f>L26/L27</f>
-        <v>734.41710270278793</v>
+        <f t="shared" si="38"/>
+        <v>816.50516372521986</v>
       </c>
       <c r="M88" s="118">
-        <f>M26/M27</f>
-        <v>1779.915399049032</v>
+        <f t="shared" si="38"/>
+        <v>1966.0518176842911</v>
       </c>
     </row>
     <row r="89" spans="2:13" ht="13" x14ac:dyDescent="0.15">
@@ -18573,44 +18573,44 @@
         <v>364</v>
       </c>
       <c r="D90" s="118">
-        <f>D62/D89</f>
-        <v>0.80895198682443781</v>
+        <f t="shared" ref="D90:M90" si="39">D62/D89</f>
+        <v>1.0653044900613822</v>
       </c>
       <c r="E90" s="118">
-        <f>E62/E89</f>
-        <v>4.494236405247559</v>
+        <f t="shared" si="39"/>
+        <v>5.1106863155835649</v>
       </c>
       <c r="F90" s="118">
-        <f>F62/F89</f>
-        <v>4.2644910722477762</v>
+        <f t="shared" si="39"/>
+        <v>4.9224288924288082</v>
       </c>
       <c r="G90" s="118">
-        <f>G62/G89</f>
-        <v>5.3754789785983643</v>
+        <f t="shared" si="39"/>
+        <v>6.1481050730758042</v>
       </c>
       <c r="H90" s="118">
-        <f>H62/H89</f>
-        <v>6.7938153926541371</v>
+        <f t="shared" si="39"/>
+        <v>7.705310216552598</v>
       </c>
       <c r="I90" s="118">
-        <f>I62/I89</f>
-        <v>8.6208663706453592</v>
+        <f t="shared" si="39"/>
+        <v>9.7025466023144791</v>
       </c>
       <c r="J90" s="118">
-        <f>J62/J89</f>
-        <v>10.98309772194906</v>
+        <f t="shared" si="39"/>
+        <v>12.274503363325364</v>
       </c>
       <c r="K90" s="118">
-        <f>K62/K89</f>
-        <v>14.13850832497668</v>
+        <f t="shared" si="39"/>
+        <v>15.697996625822482</v>
       </c>
       <c r="L90" s="118">
-        <f>L62/L89</f>
-        <v>18.450503419735949</v>
+        <f t="shared" si="39"/>
+        <v>20.362159977095107</v>
       </c>
       <c r="M90" s="118">
-        <f>M62/M89</f>
-        <v>14.502165921754102</v>
+        <f t="shared" si="39"/>
+        <v>15.915731551638485</v>
       </c>
     </row>
     <row r="91" spans="2:13" ht="13" x14ac:dyDescent="0.15">
@@ -18654,43 +18654,43 @@
         <v>366</v>
       </c>
       <c r="D92" s="118">
-        <f>D91/D32</f>
-        <v>5.550966462910953</v>
+        <f t="shared" ref="D92:M92" si="40">D91/D32</f>
+        <v>3.9749201466934818</v>
       </c>
       <c r="E92" s="118">
-        <f>E91/E32</f>
-        <v>0.6340329887364039</v>
+        <f t="shared" si="40"/>
+        <v>0.53682484210639336</v>
       </c>
       <c r="F92" s="118">
-        <f>F91/F32</f>
-        <v>0.477059962457897</v>
+        <f t="shared" si="40"/>
+        <v>0.40877809883829974</v>
       </c>
       <c r="G92" s="118">
-        <f>G91/G32</f>
-        <v>0.35539875043134411</v>
+        <f t="shared" si="40"/>
+        <v>0.30780934218288158</v>
       </c>
       <c r="H92" s="118">
-        <f>H91/H32</f>
-        <v>0.26064928638597801</v>
+        <f t="shared" si="40"/>
+        <v>0.22793441779244636</v>
       </c>
       <c r="I92" s="118">
-        <f>I91/I32</f>
-        <v>0.1866872178843462</v>
+        <f t="shared" si="40"/>
+        <v>0.16468568885592963</v>
       </c>
       <c r="J92" s="118">
-        <f>J91/J32</f>
-        <v>0.12906548119843894</v>
+        <f t="shared" si="40"/>
+        <v>0.11476053772556309</v>
       </c>
       <c r="K92" s="118">
-        <f>K91/K32</f>
-        <v>8.3859490787008661E-2</v>
+        <f t="shared" si="40"/>
+        <v>7.5105725861286693E-2</v>
       </c>
       <c r="L92" s="118">
-        <f>L91/L32</f>
-        <v>4.8497304908023432E-2</v>
+        <f t="shared" si="40"/>
+        <v>4.3723075514740542E-2</v>
       </c>
       <c r="M92" s="118">
-        <f>M91/M32</f>
+        <f t="shared" si="40"/>
         <v>0</v>
       </c>
     </row>
@@ -22371,7 +22371,7 @@
       <c r="A16" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="B16" s="165">
+      <c r="B16" s="154">
         <f>SUM(B14:K14)</f>
         <v>26880322416.543213</v>
       </c>
@@ -22670,10 +22670,10 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="161" t="s">
+      <c r="A26" s="159" t="s">
         <v>136</v>
       </c>
-      <c r="B26" s="161"/>
+      <c r="B26" s="159"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="43" t="s">
@@ -22845,22 +22845,22 @@
       <c r="D42" s="55"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A44" s="162" t="s">
+      <c r="A44" s="160" t="s">
         <v>167</v>
       </c>
-      <c r="B44" s="162"/>
-      <c r="C44" s="162"/>
-      <c r="D44" s="162"/>
-      <c r="E44" s="162"/>
-      <c r="F44" s="162"/>
-      <c r="G44" s="162"/>
-      <c r="I44" s="163"/>
-      <c r="J44" s="163"/>
-      <c r="K44" s="163"/>
-      <c r="L44" s="163"/>
-      <c r="M44" s="163"/>
-      <c r="N44" s="163"/>
-      <c r="O44" s="163"/>
+      <c r="B44" s="160"/>
+      <c r="C44" s="160"/>
+      <c r="D44" s="160"/>
+      <c r="E44" s="160"/>
+      <c r="F44" s="160"/>
+      <c r="G44" s="160"/>
+      <c r="I44" s="161"/>
+      <c r="J44" s="161"/>
+      <c r="K44" s="161"/>
+      <c r="L44" s="161"/>
+      <c r="M44" s="161"/>
+      <c r="N44" s="161"/>
+      <c r="O44" s="161"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
@@ -24185,15 +24185,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="158" t="s">
+      <c r="A1" s="162" t="s">
         <v>188</v>
       </c>
-      <c r="B1" s="158"/>
-      <c r="C1" s="158"/>
-      <c r="D1" s="158"/>
-      <c r="E1" s="158"/>
-      <c r="F1" s="158"/>
-      <c r="G1" s="158"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
       <c r="P1" s="63" t="s">
         <v>189</v>
       </c>
@@ -24205,17 +24205,17 @@
       <c r="V1" s="63"/>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A3" s="153" t="s">
+      <c r="A3" s="163" t="s">
         <v>190</v>
       </c>
-      <c r="B3" s="153"/>
+      <c r="B3" s="163"/>
       <c r="D3" s="64" t="s">
         <v>191</v>
       </c>
-      <c r="P3" s="154" t="s">
+      <c r="P3" s="164" t="s">
         <v>190</v>
       </c>
-      <c r="Q3" s="154"/>
+      <c r="Q3" s="164"/>
       <c r="S3" s="64" t="s">
         <v>191</v>
       </c>
@@ -24480,13 +24480,13 @@
         <f>AG9*AG10</f>
         <v>682.10548276114309</v>
       </c>
-      <c r="AM13" s="156" t="s">
+      <c r="AM13" s="166" t="s">
         <v>233</v>
       </c>
-      <c r="AN13" s="157"/>
-      <c r="AO13" s="157"/>
-      <c r="AP13" s="157"/>
-      <c r="AQ13" s="157"/>
+      <c r="AN13" s="167"/>
+      <c r="AO13" s="167"/>
+      <c r="AP13" s="167"/>
+      <c r="AQ13" s="167"/>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -24572,22 +24572,22 @@
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A17" s="153" t="s">
+      <c r="A17" s="163" t="s">
         <v>243</v>
       </c>
-      <c r="B17" s="153"/>
-      <c r="C17" s="153"/>
-      <c r="D17" s="153"/>
-      <c r="E17" s="153"/>
-      <c r="F17" s="153"/>
-      <c r="G17" s="153"/>
-      <c r="I17" s="153" t="s">
+      <c r="B17" s="163"/>
+      <c r="C17" s="163"/>
+      <c r="D17" s="163"/>
+      <c r="E17" s="163"/>
+      <c r="F17" s="163"/>
+      <c r="G17" s="163"/>
+      <c r="I17" s="163" t="s">
         <v>233</v>
       </c>
-      <c r="J17" s="153"/>
-      <c r="K17" s="153"/>
-      <c r="L17" s="153"/>
-      <c r="M17" s="153"/>
+      <c r="J17" s="163"/>
+      <c r="K17" s="163"/>
+      <c r="L17" s="163"/>
+      <c r="M17" s="163"/>
       <c r="P17" s="64" t="s">
         <v>244</v>
       </c>
@@ -24668,22 +24668,22 @@
       <c r="M19" s="67" t="s">
         <v>174</v>
       </c>
-      <c r="P19" s="155" t="s">
+      <c r="P19" s="165" t="s">
         <v>243</v>
       </c>
-      <c r="Q19" s="155"/>
-      <c r="R19" s="155"/>
-      <c r="S19" s="155"/>
-      <c r="T19" s="155"/>
-      <c r="U19" s="155"/>
-      <c r="V19" s="155"/>
-      <c r="X19" s="155" t="s">
+      <c r="Q19" s="165"/>
+      <c r="R19" s="165"/>
+      <c r="S19" s="165"/>
+      <c r="T19" s="165"/>
+      <c r="U19" s="165"/>
+      <c r="V19" s="165"/>
+      <c r="X19" s="165" t="s">
         <v>233</v>
       </c>
-      <c r="Y19" s="155"/>
-      <c r="Z19" s="155"/>
-      <c r="AA19" s="155"/>
-      <c r="AB19" s="155"/>
+      <c r="Y19" s="165"/>
+      <c r="Z19" s="165"/>
+      <c r="AA19" s="165"/>
+      <c r="AB19" s="165"/>
       <c r="AF19" s="72" t="s">
         <v>249</v>
       </c>
@@ -26141,13 +26141,13 @@
         <f t="shared" si="5"/>
         <v>6510</v>
       </c>
-      <c r="I32" s="153" t="s">
+      <c r="I32" s="163" t="s">
         <v>253</v>
       </c>
-      <c r="J32" s="153"/>
-      <c r="K32" s="153"/>
-      <c r="L32" s="153"/>
-      <c r="M32" s="153"/>
+      <c r="J32" s="163"/>
+      <c r="K32" s="163"/>
+      <c r="L32" s="163"/>
+      <c r="M32" s="163"/>
       <c r="P32" s="79">
         <v>11</v>
       </c>
@@ -28219,15 +28219,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="P19:V19"/>
+    <mergeCell ref="X19:AB19"/>
+    <mergeCell ref="AM13:AQ13"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="I17:M17"/>
     <mergeCell ref="I32:M32"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="P19:V19"/>
-    <mergeCell ref="X19:AB19"/>
-    <mergeCell ref="AM13:AQ13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D9" r:id="rId1" xr:uid="{FE201A1B-6C8C-4A0F-801E-10AC66BA1A74}"/>

</xml_diff>